<commit_message>
data file for driver experience
</commit_message>
<xml_diff>
--- a/Data_Dictionary.xlsx
+++ b/Data_Dictionary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimonOM\Repositories\Formula-1-Constructor-Repository\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\owens\Repositories\Formula-1-Constructor-Repository\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF65E74F-A0C0-46E8-9416-D748BF035C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B22310F-B288-443A-B5D5-710A7F845B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="1500" windowWidth="16410" windowHeight="14145" xr2:uid="{B38841E1-F419-4689-90BF-F91CA7B5FE4B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B38841E1-F419-4689-90BF-F91CA7B5FE4B}"/>
   </bookViews>
   <sheets>
     <sheet name="Data_Dictionary" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="55">
   <si>
     <t>Season</t>
   </si>
@@ -302,6 +302,12 @@
   </si>
   <si>
     <t>`Prior_Season_Grand_Prix_Wins_Last5GP` ÷ 5</t>
+  </si>
+  <si>
+    <t>The total number of Formula 1 races started by the two drivers contracted to the team at the start of the season, regardless of any mid-season driver changes.</t>
+  </si>
+  <si>
+    <t>Driver_Lineup_Experience</t>
   </si>
 </sst>
 </file>
@@ -1251,12 +1257,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8CC40D8-CCDB-4691-9AE9-BD3F7CAB3CBE}">
-  <dimension ref="A1:XFB27"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:XFB28"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="40.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="40.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29" customWidth="1"/>
-    <col min="3" max="3" width="255.7109375" customWidth="1"/>
+    <col min="3" max="3" width="255.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1494,7 +1500,7 @@
       <c r="B23" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1516,7 +1522,7 @@
       <c r="B25" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="1" t="s">
         <v>52</v>
       </c>
     </row>
@@ -9732,6 +9738,17 @@
         <v>42</v>
       </c>
     </row>
+    <row r="28" spans="1:1024 1026:2048 2050:3072 3074:4096 4098:5120 5122:6144 6146:7168 7170:8192 8194:9216 9218:10240 10242:11264 11266:12288 12290:13312 13314:14336 14338:15360 15362:16382">
+      <c r="A28" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:C1"/>

</xml_diff>

<commit_message>
data added to driver_exp file
</commit_message>
<xml_diff>
--- a/Data_Dictionary.xlsx
+++ b/Data_Dictionary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\owens\Repositories\Formula-1-Constructor-Repository\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimonOM\Repositories\Formula-1-Constructor-Repository\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B22310F-B288-443A-B5D5-710A7F845B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26218E12-5353-46EF-9951-3A3CD79047C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B38841E1-F419-4689-90BF-F91CA7B5FE4B}"/>
+    <workbookView xWindow="28800" yWindow="-11370" windowWidth="16410" windowHeight="11295" xr2:uid="{B38841E1-F419-4689-90BF-F91CA7B5FE4B}"/>
   </bookViews>
   <sheets>
     <sheet name="Data_Dictionary" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="61">
   <si>
     <t>Season</t>
   </si>
@@ -308,6 +308,24 @@
   </si>
   <si>
     <t>Driver_Lineup_Experience</t>
+  </si>
+  <si>
+    <t>Prior_Season_Quali_Avg</t>
+  </si>
+  <si>
+    <t>Average qualifying position of both team cars across all Grands Prix in the prior season.</t>
+  </si>
+  <si>
+    <t>Total number of fastest laps recorded by the team’s drivers across all Grands Prix in the prior season.</t>
+  </si>
+  <si>
+    <t>Prior_Season_Fastest_Lap_Count</t>
+  </si>
+  <si>
+    <t>Prior_Season_Fastest_Lap_Prop</t>
+  </si>
+  <si>
+    <t>Proportion of fastest laps recorded by the team’s drivers across all Grands Prix in the prior season. (`Prior_Season_Fastest_Lap_Count` ÷ `Prior_Season_Grand_Prix_Count`)</t>
   </si>
 </sst>
 </file>
@@ -1257,12 +1275,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8CC40D8-CCDB-4691-9AE9-BD3F7CAB3CBE}">
-  <dimension ref="A1:XFB28"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:XFB31"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="40.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="40.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29" customWidth="1"/>
-    <col min="3" max="3" width="255.6640625" customWidth="1"/>
+    <col min="3" max="3" width="255.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -9739,7 +9757,7 @@
       </c>
     </row>
     <row r="28" spans="1:1024 1026:2048 2050:3072 3074:4096 4098:5120 5122:6144 6146:7168 7170:8192 8194:9216 9218:10240 10242:11264 11266:12288 12290:13312 13314:14336 14338:15360 15362:16382">
-      <c r="A28" s="11" t="s">
+      <c r="A28" s="1" t="s">
         <v>54</v>
       </c>
       <c r="B28" s="1" t="s">
@@ -9747,6 +9765,39 @@
       </c>
       <c r="C28" s="1" t="s">
         <v>53</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1024 1026:2048 2050:3072 3074:4096 4098:5120 5122:6144 6146:7168 7170:8192 8194:9216 9218:10240 10242:11264 11266:12288 12290:13312 13314:14336 14338:15360 15362:16382">
+      <c r="A29" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1024 1026:2048 2050:3072 3074:4096 4098:5120 5122:6144 6146:7168 7170:8192 8194:9216 9218:10240 10242:11264 11266:12288 12290:13312 13314:14336 14338:15360 15362:16382">
+      <c r="A30" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1024 1026:2048 2050:3072 3074:4096 4098:5120 5122:6144 6146:7168 7170:8192 8194:9216 9218:10240 10242:11264 11266:12288 12290:13312 13314:14336 14338:15360 15362:16382">
+      <c r="A31" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new data dictionary variables
</commit_message>
<xml_diff>
--- a/Data_Dictionary.xlsx
+++ b/Data_Dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimonOM\Repositories\Formula-1-Constructor-Repository\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06E14A01-F666-49E4-9F75-33B2FE31F8B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECB56558-7787-4250-A35A-3424FB84467B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-12660" windowWidth="16440" windowHeight="28320" xr2:uid="{B38841E1-F419-4689-90BF-F91CA7B5FE4B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B38841E1-F419-4689-90BF-F91CA7B5FE4B}"/>
   </bookViews>
   <sheets>
     <sheet name="Data_Dictionary" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="73">
   <si>
     <t>Season</t>
   </si>
@@ -119,15 +119,6 @@
     <t>Defending_Constructor_Champ</t>
   </si>
   <si>
-    <t xml:space="preserve">The number of DNF or DNS results during the previous season (this does not include sprint race results). </t>
-  </si>
-  <si>
-    <t>Binary variable indicating whether the season included a major technical or sporting regulation change (1 = yes, 0 = no).</t>
-  </si>
-  <si>
-    <t>Numerical identifier representing a constructor’s ownership lineage across all seasons. This identifier remains constant across name, branding, or ownership transitions that preserve organizational continuity (Ex. Tyrrell → BAR → Honda → Brawn GP → Mercedes).</t>
-  </si>
-  <si>
     <t>Year in which the constructor competed in the Formula One World Championship.</t>
   </si>
   <si>
@@ -146,98 +137,10 @@
     <t>Prior_Season_NonFinish_Rate</t>
   </si>
   <si>
-    <t>The amount of points scored by a single team in the previous season (including points earned from fastest lap or sprint races).</t>
-  </si>
-  <si>
     <t>The number of Grand Prix wins by a constructor in the previous season (this does not include sprint Race wins).</t>
   </si>
   <si>
     <t>Prior_Season_Points_Earned</t>
-  </si>
-  <si>
-    <t>Constructor’s proportion of total points scored by all teams in the previous season (`Prior_Season_Points_Earned` divided by `Prior_Season_Points_Total`). This normalizes performance across seasons with different numbers of teams or scoring systems.</t>
-  </si>
-  <si>
-    <r>
-      <t>Constructor’s proportion of races won in the previous season (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>Prior_Season_Grand_Prix_Wins</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> ÷ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>Prior_Season_Grand_Prix_Count</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Constructor’s proportion of DNF or DNS results (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>Prior_Season_NonFinishes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> ÷ (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>Prior_Season_Grand_Prix_Count</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> × 2)), accounting for 2 cars per race.</t>
-    </r>
   </si>
   <si>
     <r>
@@ -292,31 +195,10 @@
     <t>Prior_Season_Win_Prop_Last5GP</t>
   </si>
   <si>
-    <t>The number of Grand Prix wins by a constructor in the previous season's first 5 rounds (this does not include sprint Race wins).</t>
-  </si>
-  <si>
-    <t>The number of Grand Prix wins by a constructor in the previous season's last 5 rounds (this does not include sprint Race wins).</t>
-  </si>
-  <si>
-    <t>`Prior_Season_Grand_Prix_Wins_First5GP` ÷ 5</t>
-  </si>
-  <si>
-    <t>`Prior_Season_Grand_Prix_Wins_Last5GP` ÷ 5</t>
-  </si>
-  <si>
-    <t>The total number of Formula 1 races started by the two drivers contracted to the team at the start of the season, regardless of any mid-season driver changes.</t>
-  </si>
-  <si>
     <t>Driver_Lineup_Experience</t>
   </si>
   <si>
     <t>Prior_Season_Quali_Avg</t>
-  </si>
-  <si>
-    <t>Average qualifying position of both team cars across all Grands Prix in the prior season.</t>
-  </si>
-  <si>
-    <t>Total number of fastest laps recorded by the team’s drivers across all Grands Prix in the prior season.</t>
   </si>
   <si>
     <t>Prior_Season_Fastest_Lap_Count</t>
@@ -325,7 +207,123 @@
     <t>Prior_Season_Fastest_Lap_Prop</t>
   </si>
   <si>
-    <t>Proportion of fastest laps recorded by the team’s drivers across all Grands Prix in the prior season. (`Prior_Season_Fastest_Lap_Count` ÷ `Prior_Season_Grand_Prix_Count`)</t>
+    <t>Grooved_Tyre_Era_Experience</t>
+  </si>
+  <si>
+    <t>Refueling_Ban_Aero_Era_Experience</t>
+  </si>
+  <si>
+    <t>Early_Turbo_Hybrid_Era_Experience</t>
+  </si>
+  <si>
+    <t>Mature_Turbo_Hybrid_Era_Experience</t>
+  </si>
+  <si>
+    <t>Ground_Effect_Era_Experience</t>
+  </si>
+  <si>
+    <t>Active_Aero_Era_Experience</t>
+  </si>
+  <si>
+    <t>Total number of Formula One World Championship race starts accumulated prior to the current season by the two drivers contracted to the constructor at the start of the season. Mid-season driver changes are not incorporated.</t>
+  </si>
+  <si>
+    <t>Total number of Formula One World Championship race starts accumulated prior to the current season within the 2026 onward regulatory era by the two drivers contracted at the start of the season.</t>
+  </si>
+  <si>
+    <t>Total number of Formula One World Championship race starts accumulated prior to the current season within the 2022 to 2025 regulatory era by the two drivers contracted at the start of the season.</t>
+  </si>
+  <si>
+    <t>Total number of Formula One World Championship race starts accumulated prior to the current season within the 2017 to 2021 regulatory era by the two drivers contracted at the start of the season.</t>
+  </si>
+  <si>
+    <t>Total number of Formula One World Championship race starts accumulated prior to the current season within the 2014 to 2016 regulatory era by the two drivers contracted at the start of the season.</t>
+  </si>
+  <si>
+    <t>Total number of Formula One World Championship race starts accumulated prior to the current season within the 2009 to 2013 regulatory era by the two drivers contracted at the start of the season.</t>
+  </si>
+  <si>
+    <t>Total number of Formula One World Championship race starts accumulated prior to the current season within the 1998 to 2008 regulatory era by the two drivers contracted at the start of the season.</t>
+  </si>
+  <si>
+    <t>Numerical identifier representing a constructor’s ownership lineage across all seasons. This identifier remains constant across name, branding, or ownership transitions that preserve competitive and organizational continuity. (Ex. Tyrrell → BAR → Honda → Brawn GP → Mercedes).</t>
+  </si>
+  <si>
+    <t>Total championship points scored by the constructor in the previous season, including points awarded for fastest lap and sprint events.</t>
+  </si>
+  <si>
+    <t>Constructor’s proportion of total points scored by all teams in the previous season. This metric normalizes performance across seasons with differing grid sizes or scoring systems.</t>
+  </si>
+  <si>
+    <r>
+      <t>Constructor’s proportion of DNF or DNS results (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Prior_Season_NonFinishes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ÷ (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Prior_Season_Grand_Prix_Count</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> × 2)), assuming two constructor entries per Grand Prix.</t>
+    </r>
+  </si>
+  <si>
+    <t>Mean qualifying position across all Grand Prix qualifying sessions for both team cars in the previous season.</t>
+  </si>
+  <si>
+    <t>The number of Grand Prix wins by a constructor in the first five rounds of the previous season, excluding sprint race wins.</t>
+  </si>
+  <si>
+    <t>The number of Grand Prix wins by a constructor in the last five rounds of the previous season, excluding sprint race wins.</t>
+  </si>
+  <si>
+    <t>The number of DNF or DNS results recorded by the constructor during the previous season, excluding sprint race results.</t>
+  </si>
+  <si>
+    <t>Binary variable indicating whether the season included a major technical or sporting regulation change as defined by the FIA (1 = yes, 0 = no).</t>
+  </si>
+  <si>
+    <t>Total number of fastest laps recorded by the team’s drivers across all Grand Prix in the prior season.</t>
+  </si>
+  <si>
+    <t>Constructor’s proportion of Grand Prix in which one of its drivers recorded the fastest lap in the previous season.</t>
+  </si>
+  <si>
+    <t>Constructor’s proportion of Grand Prix won in the previous season.</t>
+  </si>
+  <si>
+    <t>Constructor’s proportion of Grand Prix wins in the first five rounds of the previous season.</t>
+  </si>
+  <si>
+    <t>Constructor’s proportion of Grand Prix wins in the last five rounds of the previous season.</t>
   </si>
 </sst>
 </file>
@@ -513,7 +511,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="37">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -717,6 +715,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -878,7 +882,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="17" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -894,6 +898,8 @@
     <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="37" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1274,7 +1280,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8CC40D8-CCDB-4691-9AE9-BD3F7CAB3CBE}">
-  <dimension ref="A1:XFB31"/>
+  <dimension ref="A1:XFB37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.140625" bestFit="1" customWidth="1"/>
@@ -1291,7 +1297,7 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -1320,7 +1326,7 @@
         <v>14</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>30</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1331,7 +1337,7 @@
         <v>14</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1342,7 +1348,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1386,7 +1392,7 @@
         <v>14</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1397,7 +1403,7 @@
         <v>14</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1408,18 +1414,18 @@
         <v>14</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>29</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="8" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>37</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1430,7 +1436,7 @@
         <v>14</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1440,8 +1446,8 @@
       <c r="B16" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>40</v>
+      <c r="C16" s="1" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="17" spans="1:1024 1026:2048 2050:3072 3074:4096 4098:5120 5122:6144 6146:7168 7170:8192 8194:9216 9218:10240 10242:11264 11266:12288 12290:13312 13314:14336 14338:15360 15362:16382">
@@ -1452,7 +1458,7 @@
         <v>14</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:1024 1026:2048 2050:3072 3074:4096 4098:5120 5122:6144 6146:7168 7170:8192 8194:9216 9218:10240 10242:11264 11266:12288 12290:13312 13314:14336 14338:15360 15362:16382">
@@ -1474,7 +1480,7 @@
         <v>22</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>41</v>
+        <v>70</v>
       </c>
     </row>
     <row r="20" spans="1:1024 1026:2048 2050:3072 3074:4096 4098:5120 5122:6144 6146:7168 7170:8192 8194:9216 9218:10240 10242:11264 11266:12288 12290:13312 13314:14336 14338:15360 15362:16382">
@@ -1501,57 +1507,57 @@
     </row>
     <row r="22" spans="1:1024 1026:2048 2050:3072 3074:4096 4098:5120 5122:6144 6146:7168 7170:8192 8194:9216 9218:10240 10242:11264 11266:12288 12290:13312 13314:14336 14338:15360 15362:16382">
       <c r="A22" s="8" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
     </row>
     <row r="23" spans="1:1024 1026:2048 2050:3072 3074:4096 4098:5120 5122:6144 6146:7168 7170:8192 8194:9216 9218:10240 10242:11264 11266:12288 12290:13312 13314:14336 14338:15360 15362:16382">
       <c r="A23" s="1" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>51</v>
+        <v>71</v>
       </c>
     </row>
     <row r="24" spans="1:1024 1026:2048 2050:3072 3074:4096 4098:5120 5122:6144 6146:7168 7170:8192 8194:9216 9218:10240 10242:11264 11266:12288 12290:13312 13314:14336 14338:15360 15362:16382">
       <c r="A24" s="8" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>50</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:1024 1026:2048 2050:3072 3074:4096 4098:5120 5122:6144 6146:7168 7170:8192 8194:9216 9218:10240 10242:11264 11266:12288 12290:13312 13314:14336 14338:15360 15362:16382">
       <c r="A25" s="1" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
     </row>
     <row r="26" spans="1:1024 1026:2048 2050:3072 3074:4096 4098:5120 5122:6144 6146:7168 7170:8192 8194:9216 9218:10240 10242:11264 11266:12288 12290:13312 13314:14336 14338:15360 15362:16382">
-      <c r="A26" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="B26" s="1" t="s">
+      <c r="A26" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="C26" s="1" t="s">
-        <v>28</v>
+      <c r="C26" s="12" t="s">
+        <v>66</v>
       </c>
       <c r="D26" s="5"/>
       <c r="F26" s="5"/>
@@ -9745,58 +9751,124 @@
       <c r="XFB26" s="5"/>
     </row>
     <row r="27" spans="1:1024 1026:2048 2050:3072 3074:4096 4098:5120 5122:6144 6146:7168 7170:8192 8194:9216 9218:10240 10242:11264 11266:12288 12290:13312 13314:14336 14338:15360 15362:16382">
-      <c r="A27" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B27" s="1" t="s">
+      <c r="A27" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B27" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="C27" s="1" t="s">
-        <v>42</v>
+      <c r="C27" s="12" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="28" spans="1:1024 1026:2048 2050:3072 3074:4096 4098:5120 5122:6144 6146:7168 7170:8192 8194:9216 9218:10240 10242:11264 11266:12288 12290:13312 13314:14336 14338:15360 15362:16382">
       <c r="A28" s="1" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="29" spans="1:1024 1026:2048 2050:3072 3074:4096 4098:5120 5122:6144 6146:7168 7170:8192 8194:9216 9218:10240 10242:11264 11266:12288 12290:13312 13314:14336 14338:15360 15362:16382">
       <c r="A29" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="30" spans="1:1024 1026:2048 2050:3072 3074:4096 4098:5120 5122:6144 6146:7168 7170:8192 8194:9216 9218:10240 10242:11264 11266:12288 12290:13312 13314:14336 14338:15360 15362:16382">
-      <c r="A30" s="8" t="s">
-        <v>58</v>
+      <c r="A30" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="31" spans="1:1024 1026:2048 2050:3072 3074:4096 4098:5120 5122:6144 6146:7168 7170:8192 8194:9216 9218:10240 10242:11264 11266:12288 12290:13312 13314:14336 14338:15360 15362:16382">
       <c r="A31" s="1" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="B31" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1024 1026:2048 2050:3072 3074:4096 4098:5120 5122:6144 6146:7168 7170:8192 8194:9216 9218:10240 10242:11264 11266:12288 12290:13312 13314:14336 14338:15360 15362:16382">
+      <c r="A32" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C31" s="1" t="s">
-        <v>60</v>
+      <c r="C37" s="1" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated data dictionary and feature engineering
</commit_message>
<xml_diff>
--- a/Data_Dictionary.xlsx
+++ b/Data_Dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimonOM\Repositories\Formula-1-Constructor-Repository\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98F54FFB-413F-4D63-9AF8-9F350B3B191B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A07B725-68A4-488A-B979-848E55C677DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B38841E1-F419-4689-90BF-F91CA7B5FE4B}"/>
+    <workbookView xWindow="28680" yWindow="-12660" windowWidth="16440" windowHeight="28320" xr2:uid="{B38841E1-F419-4689-90BF-F91CA7B5FE4B}"/>
   </bookViews>
   <sheets>
     <sheet name="Data_Dictionary" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="93">
   <si>
     <t>Season</t>
   </si>
@@ -51,9 +51,6 @@
   </si>
   <si>
     <t>Column</t>
-  </si>
-  <si>
-    <t>Prior_Season_Points_Share</t>
   </si>
   <si>
     <t>Defending_Driver_Champ</t>
@@ -180,15 +177,9 @@
     <t>Prior_Season_Grand_Prix_Wins_First5GP</t>
   </si>
   <si>
-    <t>Prior_Season_Win_Prop_First5GP</t>
-  </si>
-  <si>
     <t>Prior_Season_Grand_Prix_Wins_Last5GP</t>
   </si>
   <si>
-    <t>Prior_Season_Win_Prop_Last5GP</t>
-  </si>
-  <si>
     <t>Prior_Season_Quali_Avg</t>
   </si>
   <si>
@@ -249,12 +240,6 @@
     <t>Constructor’s proportion of Grand Prix won in the previous season.</t>
   </si>
   <si>
-    <t>Constructor’s proportion of Grand Prix wins in the first five rounds of the previous season.</t>
-  </si>
-  <si>
-    <t>Constructor’s proportion of Grand Prix wins in the last five rounds of the previous season.</t>
-  </si>
-  <si>
     <t>Total number of laps completed in Grand Prix prior to the current season within the 1998 to 2008 regulatory era by the two drivers contracted at the start of the season.</t>
   </si>
   <si>
@@ -358,6 +343,9 @@
   </si>
   <si>
     <t>Total number of Grand Prix won within the 1998 to 2008 regulatory era by the two drivers contracted at the start of the season.</t>
+  </si>
+  <si>
+    <t>Prior_Season_Points_Prop</t>
   </si>
 </sst>
 </file>
@@ -905,7 +893,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="17" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -920,6 +908,7 @@
     <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1300,7 +1289,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8CC40D8-CCDB-4691-9AE9-BD3F7CAB3CBE}">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="47.7109375" bestFit="1" customWidth="1"/>
@@ -1310,14 +1299,14 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B2" s="9"/>
       <c r="C2" s="9"/>
@@ -1332,21 +1321,21 @@
         <v>5</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1354,10 +1343,10 @@
         <v>0</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1365,21 +1354,21 @@
         <v>1</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -1387,7 +1376,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>3</v>
@@ -1395,35 +1384,35 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -1431,406 +1420,384 @@
         <v>4</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>6</v>
+        <v>92</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
+      <c r="A22" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>37</v>
-      </c>
       <c r="B23" s="1" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="7" t="s">
-        <v>38</v>
+      <c r="A24" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>39</v>
+        <v>64</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>48</v>
+        <v>63</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>63</v>
+        <v>85</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>62</v>
+        <v>86</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>88</v>
+        <v>37</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>95</v>
+        <v>50</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" s="1" t="s">
-        <v>89</v>
+      <c r="A46" s="7" t="s">
+        <v>38</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>96</v>
+        <v>54</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
driver data - 1999
</commit_message>
<xml_diff>
--- a/Data_Dictionary.xlsx
+++ b/Data_Dictionary.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A07B725-68A4-488A-B979-848E55C677DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-12660" windowWidth="16440" windowHeight="28320" xr2:uid="{B38841E1-F419-4689-90BF-F91CA7B5FE4B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B38841E1-F419-4689-90BF-F91CA7B5FE4B}"/>
   </bookViews>
   <sheets>
     <sheet name="Data_Dictionary" sheetId="1" r:id="rId1"/>
@@ -893,7 +893,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="17" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -908,7 +908,6 @@
     <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1515,7 +1514,7 @@
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
+      <c r="A22" s="1" t="s">
         <v>35</v>
       </c>
       <c r="B22" s="1" t="s">
@@ -1526,7 +1525,7 @@
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
+      <c r="A23" s="1" t="s">
         <v>36</v>
       </c>
       <c r="B23" s="1" t="s">

</xml_diff>

<commit_message>
new variables and updated data dictionary
</commit_message>
<xml_diff>
--- a/Data_Dictionary.xlsx
+++ b/Data_Dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimonOM\Repositories\Formula-1-Constructor-Repository\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EB1C2AC-AE42-4B14-8A74-569148347384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F0EE2C0-E536-4772-A293-4C857E44668A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B38841E1-F419-4689-90BF-F91CA7B5FE4B}"/>
+    <workbookView xWindow="28680" yWindow="-12660" windowWidth="16440" windowHeight="28320" xr2:uid="{B38841E1-F419-4689-90BF-F91CA7B5FE4B}"/>
   </bookViews>
   <sheets>
     <sheet name="Data_Dictionary" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="69">
   <si>
     <t>Season</t>
   </si>
@@ -63,9 +63,6 @@
   </si>
   <si>
     <t>Prior_Season_Grand_Prix_Wins</t>
-  </si>
-  <si>
-    <t>Prior_Season_Grand_Prix_Count</t>
   </si>
   <si>
     <t>Description</t>
@@ -186,27 +183,6 @@
     <t>Prior_Season_Fastest_Lap_Prop</t>
   </si>
   <si>
-    <t>Total number of Formula One World Championship race starts accumulated prior to the current season by the two drivers contracted to the constructor at the start of the season. Mid-season driver changes are not incorporated.</t>
-  </si>
-  <si>
-    <t>Total number of Formula One World Championship race starts accumulated prior to the current season within the 2026 onward regulatory era by the two drivers contracted at the start of the season.</t>
-  </si>
-  <si>
-    <t>Total number of Formula One World Championship race starts accumulated prior to the current season within the 2022 to 2025 regulatory era by the two drivers contracted at the start of the season.</t>
-  </si>
-  <si>
-    <t>Total number of Formula One World Championship race starts accumulated prior to the current season within the 2017 to 2021 regulatory era by the two drivers contracted at the start of the season.</t>
-  </si>
-  <si>
-    <t>Total number of Formula One World Championship race starts accumulated prior to the current season within the 2014 to 2016 regulatory era by the two drivers contracted at the start of the season.</t>
-  </si>
-  <si>
-    <t>Total number of Formula One World Championship race starts accumulated prior to the current season within the 2009 to 2013 regulatory era by the two drivers contracted at the start of the season.</t>
-  </si>
-  <si>
-    <t>Total number of Formula One World Championship race starts accumulated prior to the current season within the 1998 to 2008 regulatory era by the two drivers contracted at the start of the season.</t>
-  </si>
-  <si>
     <t>Numerical identifier representing a constructor’s ownership lineage across all seasons. This identifier remains constant across name, branding, or ownership transitions that preserve competitive and organizational continuity. (Ex. Tyrrell → BAR → Honda → Brawn GP → Mercedes).</t>
   </si>
   <si>
@@ -237,111 +213,12 @@
     <t>Constructor’s proportion of Grand Prix won in the previous season.</t>
   </si>
   <si>
-    <t>Total number of laps completed in Grand Prix prior to the current season within the 1998 to 2008 regulatory era by the two drivers contracted at the start of the season.</t>
-  </si>
-  <si>
-    <t>Total number of laps completed in Grand Prix prior to the current season within the 2009 to 2013 regulatory era by the two drivers contracted at the start of the season.</t>
-  </si>
-  <si>
-    <t>Total number of laps completed in Grand Prix prior to the current season within the 2014 to 2016 regulatory era by the two drivers contracted at the start of the season.</t>
-  </si>
-  <si>
-    <t>Total number of laps completed in Grand Prix prior to the current season within the 2017 to 2021 regulatory era by the two drivers contracted at the start of the season.</t>
-  </si>
-  <si>
-    <t>Total number of laps completed in Grand Prix prior to the current season within the 2022 to 2025 regulatory era by the two drivers contracted at the start of the season.</t>
-  </si>
-  <si>
-    <t>Total number of laps completed in Grand Prix prior to the current season within the 2026 onward regulatory era by the two drivers contracted at the start of the season.</t>
-  </si>
-  <si>
     <t>Total number of laps completed in Grand Prix prior to the current season by the two drivers contracted to the constructor at the start of the season. Mid-season driver changes are not incorporated.</t>
   </si>
   <si>
-    <t>Driver_Lineup_Experience_Active_Aero_Era</t>
-  </si>
-  <si>
-    <t>Driver_Lineup_Experience_Ground_Effect_Era</t>
-  </si>
-  <si>
-    <t>Driver_Lineup_Total_Experience</t>
-  </si>
-  <si>
-    <t>Driver_Lineup_Experience_Mature_Turbo_Hybrid_Era</t>
-  </si>
-  <si>
-    <t>Driver_Lineup_Experience_Early_Turbo_Hybrid_Era</t>
-  </si>
-  <si>
-    <t>Driver_Lineup_Experience_Refueling_Ban_Aero_Era</t>
-  </si>
-  <si>
-    <t>Driver_Lineup_Experience_Grooved_Tyre_Era</t>
-  </si>
-  <si>
     <t>Driver_Lineup_Total_Laps_Completed</t>
   </si>
   <si>
-    <t>Driver_Lineup_Laps_Active_Aero_Era</t>
-  </si>
-  <si>
-    <t>Driver_Lineup_Laps_Ground_Effect_Era</t>
-  </si>
-  <si>
-    <t>Driver_Lineup_Laps_Mature_Turbo_Hybrid_Era</t>
-  </si>
-  <si>
-    <t>Driver_Lineup_Laps_Early_Turbo_Hybrid_Era</t>
-  </si>
-  <si>
-    <t>Driver_Lineup_Laps_Refueling_Ban_Aero_Era</t>
-  </si>
-  <si>
-    <t>Driver_Lineup_Laps_Grooved_Tyre_Era</t>
-  </si>
-  <si>
-    <t>Driver_Lineup_Total_Wins</t>
-  </si>
-  <si>
-    <t>Driver_Lineup_Wins_Active_Aero_Era</t>
-  </si>
-  <si>
-    <t>Driver_Lineup_Wins_Ground_Effect_Era</t>
-  </si>
-  <si>
-    <t>Driver_Lineup_Wins_Mature_Turbo_Hybrid_Era</t>
-  </si>
-  <si>
-    <t>Driver_Lineup_Wins_Early_Turbo_Hybrid_Era</t>
-  </si>
-  <si>
-    <t>Driver_Lineup_Wins_Refueling_Ban_Aero_Era</t>
-  </si>
-  <si>
-    <t>Driver_Lineup_Wins_Grooved_Tyre_Era</t>
-  </si>
-  <si>
-    <t>Total number of career Grand Prix wins achieved by the two drivers contracted to the constructor at the start of the season. Mid-season driver changes are not incorporated.</t>
-  </si>
-  <si>
-    <t>Total number of Grand Prix won within the 2026 onward regulatory era by the two drivers contracted at the start of the season.</t>
-  </si>
-  <si>
-    <t>Total number of Grand Prix won within the 2022 to 2025 regulatory era by the two drivers contracted at the start of the season.</t>
-  </si>
-  <si>
-    <t>Total number of Grand Prix won within the 2017 to 2021 regulatory era by the two drivers contracted at the start of the season.</t>
-  </si>
-  <si>
-    <t>Total number of Grand Prix won within the 2014 to 2026 regulatory era by the two drivers contracted at the start of the season.</t>
-  </si>
-  <si>
-    <t>Total number of Grand Prix won within the 2009 to 2013 regulatory era by the two drivers contracted at the start of the season.</t>
-  </si>
-  <si>
-    <t>Total number of Grand Prix won within the 1998 to 2008 regulatory era by the two drivers contracted at the start of the season.</t>
-  </si>
-  <si>
     <t>Prior_Season_Points_Prop</t>
   </si>
   <si>
@@ -352,6 +229,51 @@
   </si>
   <si>
     <t>Binary variable indicating whether the constructor’s primary factory operations (not nationality, not engine supplier) are based in the United Kingdom (1 = factory in the United Kingdom, 0 = factory not in the United Kingdom).</t>
+  </si>
+  <si>
+    <t>Driver_Lineup_Total_Race_Starts</t>
+  </si>
+  <si>
+    <t>Driver_Lineup_3_Season_Laps_Completed</t>
+  </si>
+  <si>
+    <t>Driver_Lineup_3_Season_Laps_Prop</t>
+  </si>
+  <si>
+    <t>Total number of laps completed in Grand Prix by both drivers over the previous 3 seasons.</t>
+  </si>
+  <si>
+    <t>Maximum possible laps for a single car across all Grand Prix in the previous 3 seasons.</t>
+  </si>
+  <si>
+    <t>Driver_Lineup_3_Season_Race_Starts</t>
+  </si>
+  <si>
+    <t>Total number of Grand Prix race starts completed by both drivers over the previous 3 seasons.</t>
+  </si>
+  <si>
+    <t>Maximum possible race starts for a single driver across all Grand Prix in the previous 3 seasons.</t>
+  </si>
+  <si>
+    <t>Driver_Lineup_3_Season_Race_Start_Prop</t>
+  </si>
+  <si>
+    <t>Total number of Formula One Grand Prix starts accumulated prior to the current season by the two drivers contracted to the constructor at the start of the season. Mid-season driver changes are not incorporated.</t>
+  </si>
+  <si>
+    <t>Prior_Season_GP_Count</t>
+  </si>
+  <si>
+    <t>Prior_3_Season_GP_Count</t>
+  </si>
+  <si>
+    <t>Prior_3_Season_Lap_Count</t>
+  </si>
+  <si>
+    <t>Proportion of total possible laps completed by the team’s two drivers over the previous 3 seasons: Driver_Lineup_3_Season_Laps_Completed ÷ (Prior_3_Season_Lap_Count x 2)</t>
+  </si>
+  <si>
+    <t>Proportion of total possible race starts completed by the team’s two drivers over the previous 3 seasons: Driver_Lineup_3_Season_Race_Starts ÷ (Prior_3_Season_GP_Count x 2)</t>
   </si>
 </sst>
 </file>
@@ -1294,7 +1216,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8CC40D8-CCDB-4691-9AE9-BD3F7CAB3CBE}">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="47.7109375" bestFit="1" customWidth="1"/>
@@ -1304,14 +1226,14 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B2" s="9"/>
       <c r="C2" s="9"/>
@@ -1326,21 +1248,21 @@
         <v>5</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1348,10 +1270,10 @@
         <v>0</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1359,21 +1281,21 @@
         <v>1</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -1381,7 +1303,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>3</v>
@@ -1389,46 +1311,46 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>93</v>
+        <v>52</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>94</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -1436,21 +1358,21 @@
         <v>4</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -1458,21 +1380,21 @@
         <v>8</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>91</v>
+        <v>50</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -1480,21 +1402,21 @@
         <v>9</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>10</v>
+        <v>64</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -1502,10 +1424,10 @@
         <v>7</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -1513,307 +1435,164 @@
         <v>6</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>64</v>
-      </c>
       <c r="B27" s="1" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>92</v>
+        <v>19</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>42</v>
+        <v>68</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>68</v>
+      <c r="A30" s="7" t="s">
+        <v>55</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>69</v>
+      <c r="A31" s="7" t="s">
+        <v>66</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>92</v>
+        <v>19</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>71</v>
+        <v>35</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
-        <v>72</v>
+      <c r="A34" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>73</v>
+        <v>37</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>92</v>
+        <v>19</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
supplementary datasets and updated feature engineering
</commit_message>
<xml_diff>
--- a/Data_Dictionary.xlsx
+++ b/Data_Dictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimonOM\Repositories\Formula-1-Constructor-Repository\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F0EE2C0-E536-4772-A293-4C857E44668A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E7FBC33-6558-4E58-BE92-EF81D6043099}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-12660" windowWidth="16440" windowHeight="28320" xr2:uid="{B38841E1-F419-4689-90BF-F91CA7B5FE4B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B38841E1-F419-4689-90BF-F91CA7B5FE4B}"/>
   </bookViews>
   <sheets>
     <sheet name="Data_Dictionary" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="71">
   <si>
     <t>Season</t>
   </si>
@@ -274,6 +274,12 @@
   </si>
   <si>
     <t>Proportion of total possible race starts completed by the team’s two drivers over the previous 3 seasons: Driver_Lineup_3_Season_Race_Starts ÷ (Prior_3_Season_GP_Count x 2)</t>
+  </si>
+  <si>
+    <t>race_starts.csv</t>
+  </si>
+  <si>
+    <t>laps_completed.csv</t>
   </si>
 </sst>
 </file>
@@ -1479,7 +1485,7 @@
         <v>54</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>63</v>
@@ -1490,7 +1496,7 @@
         <v>59</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>60</v>
@@ -1523,7 +1529,7 @@
         <v>49</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>48</v>
@@ -1534,7 +1540,7 @@
         <v>55</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>57</v>

</xml_diff>

<commit_message>
adding driver names to raw data file
</commit_message>
<xml_diff>
--- a/Data_Dictionary.xlsx
+++ b/Data_Dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimonOM\Repositories\Formula-1-Constructor-Repository\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E7FBC33-6558-4E58-BE92-EF81D6043099}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00ED48C4-4195-4A9A-8ECA-B97EB4BCDE1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B38841E1-F419-4689-90BF-F91CA7B5FE4B}"/>
+    <workbookView xWindow="28800" yWindow="-8640" windowWidth="16410" windowHeight="15480" xr2:uid="{B38841E1-F419-4689-90BF-F91CA7B5FE4B}"/>
   </bookViews>
   <sheets>
     <sheet name="Data_Dictionary" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="75">
   <si>
     <t>Season</t>
   </si>
@@ -50,9 +50,6 @@
     <t>Reg_Change_Year</t>
   </si>
   <si>
-    <t>Column</t>
-  </si>
-  <si>
     <t>Defending_Driver_Champ</t>
   </si>
   <si>
@@ -71,9 +68,6 @@
     <t>ID</t>
   </si>
   <si>
-    <t>Origin</t>
-  </si>
-  <si>
     <t>Constructor_Lineage_ID</t>
   </si>
   <si>
@@ -87,9 +81,6 @@
   </si>
   <si>
     <t>The number of Grand Prix held in the previous season (this does not include sprint races).</t>
-  </si>
-  <si>
-    <t>All prior season performance variables reflect results from the immediately preceding season and are used to simulate preseason championship prediction without incorporating in season outcomes.</t>
   </si>
   <si>
     <t>Engineered feature</t>
@@ -280,6 +271,27 @@
   </si>
   <si>
     <t>laps_completed.csv</t>
+  </si>
+  <si>
+    <t>Variable</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Driver_A</t>
+  </si>
+  <si>
+    <t>Driver_B</t>
+  </si>
+  <si>
+    <t>Name of one driver signed by the team for the current season.</t>
+  </si>
+  <si>
+    <t>Returning_Driver_Lineup</t>
+  </si>
+  <si>
+    <t>Binary variable indicating whether a constructor's driver lineup is the same as the previous season (1 = both drivers returning from previous season, 0 = at least one new driver signed with the team).</t>
   </si>
 </sst>
 </file>
@@ -1222,389 +1234,414 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8CC40D8-CCDB-4691-9AE9-BD3F7CAB3CBE}">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="47.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="255.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
+      <c r="A3" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="3" t="s">
+      <c r="A4" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>26</v>
-      </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>14</v>
+      <c r="A8" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>3</v>
+      <c r="A9" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>51</v>
+        <v>13</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>28</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>51</v>
+        <v>4</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>27</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>44</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>7</v>
+        <v>48</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>47</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>6</v>
+        <v>48</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>51</v>
+        <v>31</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>43</v>
+        <v>72</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="7" t="s">
-        <v>59</v>
+      <c r="A26" s="1" t="s">
+        <v>48</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="7" t="s">
-        <v>65</v>
+      <c r="A27" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>51</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>19</v>
+        <v>66</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>56</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>70</v>
+        <v>48</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>62</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="7" t="s">
-        <v>55</v>
+      <c r="A30" s="1" t="s">
+        <v>16</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="7" t="s">
-        <v>66</v>
+      <c r="A31" s="1" t="s">
+        <v>67</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>19</v>
+        <v>67</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>52</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>63</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>41</v>
+        <v>55</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="7" t="s">
-        <v>36</v>
+      <c r="A34" s="1" t="s">
+        <v>16</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>46</v>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
driver data - 2004
</commit_message>
<xml_diff>
--- a/Data_Dictionary.xlsx
+++ b/Data_Dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimonOM\Repositories\Formula-1-Constructor-Repository\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84F53185-C9CF-4806-9323-5F3DC1275E06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77D168C4-0344-4848-A18E-BD9784B0B76D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-12660" windowWidth="16440" windowHeight="28320" xr2:uid="{B38841E1-F419-4689-90BF-F91CA7B5FE4B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B38841E1-F419-4689-90BF-F91CA7B5FE4B}"/>
   </bookViews>
   <sheets>
     <sheet name="Data_Dictionary" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="73">
   <si>
     <t>Season</t>
   </si>
@@ -45,9 +45,6 @@
   </si>
   <si>
     <t>Target variable indicating whether a constructor won the Formula One World Championship (1 = won championship, 0 = did not win championship).</t>
-  </si>
-  <si>
-    <t>Reg_Change_Year</t>
   </si>
   <si>
     <t>Defending_Driver_Champ</t>
@@ -190,9 +187,6 @@
   </si>
   <si>
     <t>The number of Grand Prix wins by a constructor in the last five rounds of the previous season, excluding sprint race wins.</t>
-  </si>
-  <si>
-    <t>Binary variable indicating whether the season included a major technical or sporting regulation change as defined by the FIA (1 = yes, 0 = no).</t>
   </si>
   <si>
     <t>Total number of fastest laps recorded by the team’s drivers across all Grand Prix in the prior season.</t>
@@ -1234,7 +1228,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8CC40D8-CCDB-4691-9AE9-BD3F7CAB3CBE}">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" bestFit="1" customWidth="1"/>
@@ -1244,7 +1238,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -1256,62 +1250,62 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>0</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B6" s="8" t="s">
         <v>1</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>2</v>
@@ -1322,150 +1316,150 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>4</v>
+        <v>46</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>26</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B15" s="7" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>47</v>
-      </c>
       <c r="C16" s="1" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>8</v>
+        <v>59</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>61</v>
+        <v>15</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>15</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>30</v>
@@ -1476,29 +1470,29 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>40</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B24" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>71</v>
@@ -1509,134 +1503,123 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>73</v>
+        <v>49</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>51</v>
+        <v>64</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>54</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="B28" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>62</v>
+        <v>15</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>57</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>16</v>
+        <v>65</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>46</v>
+        <v>65</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>50</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B33" s="7" t="s">
-        <v>63</v>
+        <v>15</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>51</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>64</v>
+        <v>37</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B35" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B35" s="7" t="s">
         <v>32</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B36" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>